<commit_message>
FY26: Excel-driven business model and forecasts; home title rebrand
- Load Digital_Platforms_Business_Model.xlsx via dev middleware and exported JSON;
  parse Current Model Growth for live table and forecast metrics on Digital Apps playbook.
- Add bridge from sheet grids to funnel/chart data; Fy26ForecastMetricsContext for FY26 UI.
- Export digital-platforms-business-model.json in export-roadmaps; extend Vite local-data route.
- Rename home page H1 and index title to Digital Experience and Solutions.
- Update workbook and SkyportCare roadmap exports.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/Digital_Platforms_Business_Model.xlsx
+++ b/Digital_Platforms_Business_Model.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goodmanglobal-my.sharepoint.com/personal/ganesvx_daikincomfort_com/Documents/Lee/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vishwas/Documents/DevelopmentProjects/Skyport-Web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1001" documentId="13_ncr:1_{1748F867-2406-954C-B76E-BFD6231F8FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B79D303-943F-4F46-87EC-59E739840120}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A991CD-BD5B-CD41-A13D-7CB9ABE7FAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3020" yWindow="640" windowWidth="30060" windowHeight="23760" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="180" yWindow="760" windowWidth="30060" windowHeight="17760" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Old - Do Not Use" sheetId="7" r:id="rId1"/>

</xml_diff>